<commit_message>
fix: Smart Skip algoritması tam eşleşmeye çevrildi. Fractal ve HP Filter hataları temizlendi. Data botu Adjusted Close ve doğru path'e ayarlandı. main.py sonuna otomatik Master Rapor oluşturucu eklendi.
</commit_message>
<xml_diff>
--- a/vbt_bist/output/AKBNK/AKBNK_Karsilastirma.xlsx
+++ b/vbt_bist/output/AKBNK/AKBNK_Karsilastirma.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,7 +445,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>103.42</v>
+        <v>104.03</v>
       </c>
     </row>
     <row r="3">
@@ -460,7 +460,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>88.63</v>
+        <v>92.13</v>
       </c>
     </row>
     <row r="4">
@@ -471,11 +471,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>zlema</t>
+          <t>tsi</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>87.63</v>
+        <v>86.27</v>
       </c>
     </row>
     <row r="5">
@@ -486,11 +486,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>psar</t>
+          <t>zlema</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>77.64</v>
+        <v>77.67</v>
       </c>
     </row>
     <row r="6">
@@ -501,11 +501,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tsi</t>
+          <t>psar</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>67.62</v>
+        <v>66.36</v>
       </c>
     </row>
     <row r="7">
@@ -576,11 +576,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>bollinger</t>
+          <t>ppo</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>51.44</v>
+        <v>53.83</v>
       </c>
     </row>
     <row r="12">
@@ -591,11 +591,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>macd</t>
+          <t>adx_macd</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>51.39</v>
+        <v>48.25</v>
       </c>
     </row>
     <row r="13">
@@ -606,11 +606,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>tema</t>
+          <t>macd</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>50.19</v>
+        <v>46.88</v>
       </c>
     </row>
     <row r="14">
@@ -621,11 +621,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>adx_macd</t>
+          <t>alma</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>48.25</v>
+        <v>46.52</v>
       </c>
     </row>
     <row r="15">
@@ -666,11 +666,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>alma</t>
+          <t>historical_vol_rank</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>43.8</v>
+        <v>45.01</v>
       </c>
     </row>
     <row r="18">
@@ -681,11 +681,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ppo</t>
+          <t>williams_r</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>37.17</v>
+        <v>37.05</v>
       </c>
     </row>
     <row r="19">
@@ -696,11 +696,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>williams_r</t>
+          <t>bollinger</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>36.64</v>
+        <v>36.68</v>
       </c>
     </row>
     <row r="20">
@@ -711,11 +711,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>single_ma</t>
+          <t>elder_ray</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>35.76</v>
+        <v>35.95</v>
       </c>
     </row>
     <row r="21">
@@ -741,11 +741,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>historical_vol_rank</t>
+          <t>tema</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>34.69</v>
+        <v>31.59</v>
       </c>
     </row>
     <row r="23">
@@ -756,11 +756,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>mfi</t>
+          <t>chandelier</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>31.9</v>
+        <v>30.83</v>
       </c>
     </row>
     <row r="24">
@@ -771,11 +771,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>chandelier</t>
+          <t>vwap</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>30.83</v>
+        <v>30.01</v>
       </c>
     </row>
     <row r="25">
@@ -786,11 +786,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>vwap</t>
+          <t>klinger</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>30.01</v>
+        <v>29.34</v>
       </c>
     </row>
     <row r="26">
@@ -801,11 +801,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>mass_index</t>
+          <t>single_ma</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>27.33</v>
+        <v>29.24</v>
       </c>
     </row>
     <row r="27">
@@ -816,11 +816,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>vwma</t>
+          <t>chaikin_vol</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>26.78</v>
+        <v>28.06</v>
       </c>
     </row>
     <row r="28">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>26.75</v>
+        <v>27.95</v>
       </c>
     </row>
     <row r="29">
@@ -846,11 +846,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>rsi</t>
+          <t>mass_index</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26.31</v>
+        <v>27.33</v>
       </c>
     </row>
     <row r="30">
@@ -861,11 +861,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>roc</t>
+          <t>vwma</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>26.25</v>
+        <v>26.78</v>
       </c>
     </row>
     <row r="31">
@@ -891,11 +891,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>supertrend</t>
+          <t>roc</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.58</v>
+        <v>25.95</v>
       </c>
     </row>
     <row r="33">
@@ -906,11 +906,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>chaikin_vol</t>
+          <t>supertrend</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>24.2</v>
+        <v>25.58</v>
       </c>
     </row>
     <row r="34">
@@ -921,11 +921,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>fractal_breakout</t>
+          <t>vpt</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>23.04</v>
+        <v>23.46</v>
       </c>
     </row>
     <row r="35">
@@ -936,11 +936,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>coppock</t>
+          <t>ad_line</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>21.49</v>
+        <v>19.69</v>
       </c>
     </row>
     <row r="36">
@@ -966,11 +966,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>klinger</t>
+          <t>mfi</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>18.7</v>
+        <v>19.05</v>
       </c>
     </row>
     <row r="38">
@@ -981,11 +981,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>elder_ray</t>
+          <t>coppock</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>18.52</v>
+        <v>18.23</v>
       </c>
     </row>
     <row r="39">
@@ -996,11 +996,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>vpt</t>
+          <t>std_channel</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>18.24</v>
+        <v>18.16</v>
       </c>
     </row>
     <row r="40">
@@ -1011,11 +1011,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>std_channel</t>
+          <t>cci</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>18.16</v>
+        <v>15.12</v>
       </c>
     </row>
     <row r="41">
@@ -1026,11 +1026,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>aroon</t>
+          <t>rsi</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>15.39</v>
+        <v>14</v>
       </c>
     </row>
     <row r="42">
@@ -1041,11 +1041,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>schaff_trend</t>
+          <t>atr_channel</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>14.25</v>
+        <v>11.58</v>
       </c>
     </row>
     <row r="43">
@@ -1056,11 +1056,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ad_line</t>
+          <t>schaff_trend</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>12.39</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="44">
@@ -1101,11 +1101,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>heikin_ashi</t>
+          <t>aroon</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>6.42</v>
+        <v>6.81</v>
       </c>
     </row>
     <row r="47">
@@ -1120,7 +1120,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>5.85</v>
+        <v>6.58</v>
       </c>
     </row>
     <row r="48">
@@ -1131,11 +1131,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>cci</t>
+          <t>heikin_ashi</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>5.12</v>
+        <v>6.42</v>
       </c>
     </row>
     <row r="49">
@@ -1146,11 +1146,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>stoch_rsi</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>4.77</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="50">
@@ -1161,11 +1161,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>stoch_rsi</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2.01</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="51">
@@ -1176,11 +1176,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>engulfing</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1.59</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="52">
@@ -1191,11 +1191,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>connors_rsi</t>
+          <t>fractal_breakout</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1.15</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="53">
@@ -1206,11 +1206,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>engulfing</t>
+          <t>rsi_divergence</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.92</v>
+        <v>-2.39</v>
       </c>
     </row>
     <row r="54">
@@ -1221,11 +1221,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>zscore</t>
+          <t>three_ma</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0.08</v>
+        <v>-2.69</v>
       </c>
     </row>
     <row r="55">
@@ -1236,11 +1236,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>atr_channel</t>
+          <t>bb_rsi</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>-0.19</v>
+        <v>-3.43</v>
       </c>
     </row>
     <row r="56">
@@ -1251,11 +1251,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>rsi_divergence</t>
+          <t>cmf</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>-2.39</v>
+        <v>-3.68</v>
       </c>
     </row>
     <row r="57">
@@ -1266,11 +1266,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>three_ma</t>
+          <t>awesome_oscillator</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>-2.69</v>
+        <v>-3.88</v>
       </c>
     </row>
     <row r="58">
@@ -1281,11 +1281,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>bb_rsi</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>-3.43</v>
+        <v>-5.44</v>
       </c>
     </row>
     <row r="59">
@@ -1296,11 +1296,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>cmf</t>
+          <t>connors_rsi</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>-3.68</v>
+        <v>-6.61</v>
       </c>
     </row>
     <row r="60">
@@ -1311,11 +1311,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>doji_reversal</t>
+          <t>two_ma</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>-4.67</v>
+        <v>-7.11</v>
       </c>
     </row>
     <row r="61">
@@ -1326,11 +1326,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>two_ma</t>
+          <t>obv_ma</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>-7.11</v>
+        <v>-7.42</v>
       </c>
     </row>
     <row r="62">
@@ -1341,11 +1341,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>obv_ma</t>
+          <t>squeeze</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>-7.42</v>
+        <v>-7.49</v>
       </c>
     </row>
     <row r="63">
@@ -1356,11 +1356,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>squeeze</t>
+          <t>adx</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>-7.49</v>
+        <v>-9.220000000000001</v>
       </c>
     </row>
     <row r="64">
@@ -1371,11 +1371,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>pin_bar</t>
+          <t>zscore</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>-9.9</v>
+        <v>-9.67</v>
       </c>
     </row>
     <row r="65">
@@ -1386,11 +1386,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>nvi</t>
+          <t>pin_bar</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>-11.07</v>
+        <v>-9.9</v>
       </c>
     </row>
     <row r="66">
@@ -1401,11 +1401,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>adx</t>
+          <t>nvi</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>-14.4</v>
+        <v>-11.07</v>
       </c>
     </row>
     <row r="67">
@@ -1416,11 +1416,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>obv</t>
+          <t>doji_reversal</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>-14.81</v>
+        <v>-12.31</v>
       </c>
     </row>
     <row r="68">
@@ -1431,11 +1431,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>golden_cross</t>
+          <t>obv</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>-15.41</v>
+        <v>-14.81</v>
       </c>
     </row>
     <row r="69">
@@ -1446,11 +1446,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>trend_intensity</t>
+          <t>golden_cross</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>-16.05</v>
+        <v>-15.41</v>
       </c>
     </row>
     <row r="70">
@@ -1461,11 +1461,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>awesome_oscillator</t>
+          <t>trend_intensity</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>-18.12</v>
+        <v>-16.05</v>
       </c>
     </row>
     <row r="71">
@@ -1476,11 +1476,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>eom</t>
+          <t>ema_cross</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>-18.21</v>
+        <v>-17.14</v>
       </c>
     </row>
     <row r="72">
@@ -1491,11 +1491,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ichimoku</t>
+          <t>eom</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>-18.33</v>
+        <v>-17.65</v>
       </c>
     </row>
     <row r="73">
@@ -1506,11 +1506,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>natr</t>
+          <t>linreg</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>-18.91</v>
+        <v>-17.7</v>
       </c>
     </row>
     <row r="74">
@@ -1521,11 +1521,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ema_cross</t>
+          <t>natr</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>-21.48</v>
+        <v>-18.91</v>
       </c>
     </row>
     <row r="75">
@@ -1536,11 +1536,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>linreg</t>
+          <t>true_range_ema</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>-21.92</v>
+        <v>-22.28</v>
       </c>
     </row>
     <row r="76">
@@ -1551,11 +1551,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>donchian</t>
+          <t>trix</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>-23.34</v>
+        <v>-22.5</v>
       </c>
     </row>
     <row r="77">
@@ -1566,11 +1566,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>rvi</t>
+          <t>hp_filter_ma</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>-23.5</v>
+        <v>-22.52</v>
       </c>
     </row>
     <row r="78">
@@ -1581,11 +1581,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>wma</t>
+          <t>rvi</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>-24.47</v>
+        <v>-23.5</v>
       </c>
     </row>
     <row r="79">
@@ -1596,11 +1596,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>supertrend_rsi</t>
+          <t>ichimoku</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>-25.46</v>
+        <v>-23.68</v>
       </c>
     </row>
     <row r="80">
@@ -1611,11 +1611,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>trix</t>
+          <t>wma</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>-28.77</v>
+        <v>-24.47</v>
       </c>
     </row>
     <row r="81">
@@ -1626,11 +1626,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>inside_bar</t>
+          <t>donchian</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>-29.01</v>
+        <v>-25.36</v>
       </c>
     </row>
     <row r="82">
@@ -1641,11 +1641,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>rsi_macd</t>
+          <t>supertrend_rsi</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>-30.22</v>
+        <v>-25.46</v>
       </c>
     </row>
     <row r="83">
@@ -1656,11 +1656,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>bb_width</t>
+          <t>inside_bar</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>-30.93</v>
+        <v>-29.01</v>
       </c>
     </row>
     <row r="84">
@@ -1671,11 +1671,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>vix_fix</t>
+          <t>rsi_macd</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>-33.36</v>
+        <v>-30.22</v>
       </c>
     </row>
     <row r="85">
@@ -1686,11 +1686,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>marubozu</t>
+          <t>bb_width</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>-34.92</v>
+        <v>-30.93</v>
       </c>
     </row>
     <row r="86">
@@ -1701,11 +1701,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>keltner</t>
+          <t>vix_fix</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>-36.53</v>
+        <v>-33.36</v>
       </c>
     </row>
     <row r="87">
@@ -1716,11 +1716,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>true_range_ema</t>
+          <t>marubozu</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>-37.76</v>
+        <v>-34.92</v>
       </c>
     </row>
     <row r="88">
@@ -1731,11 +1731,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>ichimoku_rsi</t>
+          <t>keltner</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>-38.64</v>
+        <v>-36.53</v>
       </c>
     </row>
     <row r="89">
@@ -1746,11 +1746,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>three_soldiers</t>
+          <t>ichimoku_rsi</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>-40.16</v>
+        <v>-38.64</v>
       </c>
     </row>
     <row r="90">
@@ -1761,11 +1761,26 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
+          <t>three_soldiers</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>-40.16</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>AKBNK</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
           <t>ibs</t>
         </is>
       </c>
-      <c r="C90" t="n">
-        <v>-58.71</v>
+      <c r="C91" t="n">
+        <v>-53.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add ffill/bfill data validation layer and run tests
</commit_message>
<xml_diff>
--- a/vbt_bist/output/AKBNK/AKBNK_Karsilastirma.xlsx
+++ b/vbt_bist/output/AKBNK/AKBNK_Karsilastirma.xlsx
@@ -816,11 +816,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>chaikin_vol</t>
+          <t>dpo</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>28.06</v>
+        <v>27.95</v>
       </c>
     </row>
     <row r="28">
@@ -831,11 +831,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>dpo</t>
+          <t>chaikin_vol</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>27.95</v>
+        <v>27.68</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
feat: Add full dashboard architecture, bug fixes and updated academic metrics
</commit_message>
<xml_diff>
--- a/vbt_bist/output/AKBNK/AKBNK_Karsilastirma.xlsx
+++ b/vbt_bist/output/AKBNK/AKBNK_Karsilastirma.xlsx
@@ -445,7 +445,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>104.03</v>
+        <v>100.58</v>
       </c>
     </row>
     <row r="3">
@@ -460,7 +460,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>92.13</v>
+        <v>88.88</v>
       </c>
     </row>
     <row r="4">
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>86.27</v>
+        <v>85.72</v>
       </c>
     </row>
     <row r="5">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>77.67</v>
+        <v>74.67</v>
       </c>
     </row>
     <row r="6">
@@ -531,11 +531,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>hma</t>
+          <t>adx_macd</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>59.29</v>
+        <v>61.61</v>
       </c>
     </row>
     <row r="9">
@@ -546,11 +546,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>triple_screen</t>
+          <t>macd</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>59.09</v>
+        <v>60.12</v>
       </c>
     </row>
     <row r="10">
@@ -561,11 +561,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>morning_star</t>
+          <t>hma</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>54.07</v>
+        <v>59.29</v>
       </c>
     </row>
     <row r="11">
@@ -576,11 +576,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ppo</t>
+          <t>triple_screen</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>53.83</v>
+        <v>56.4</v>
       </c>
     </row>
     <row r="12">
@@ -591,11 +591,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>adx_macd</t>
+          <t>morning_star</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>48.25</v>
+        <v>54.07</v>
       </c>
     </row>
     <row r="13">
@@ -606,11 +606,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>macd</t>
+          <t>ppo</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>46.88</v>
+        <v>53.37</v>
       </c>
     </row>
     <row r="14">
@@ -621,11 +621,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>alma</t>
+          <t>bollinger</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>46.52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15">
@@ -636,11 +636,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>volatility_breakout</t>
+          <t>hist_vol</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>45.76</v>
+        <v>45.51</v>
       </c>
     </row>
     <row r="16">
@@ -651,11 +651,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>hist_vol</t>
+          <t>historical_vol_rank</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>45.51</v>
+        <v>45.01</v>
       </c>
     </row>
     <row r="17">
@@ -666,11 +666,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>historical_vol_rank</t>
+          <t>alma</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>45.01</v>
+        <v>44.05</v>
       </c>
     </row>
     <row r="18">
@@ -681,11 +681,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>williams_r</t>
+          <t>volatility_breakout</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>37.05</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="19">
@@ -696,11 +696,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>bollinger</t>
+          <t>chaikin_vol</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>36.68</v>
+        <v>39.18</v>
       </c>
     </row>
     <row r="20">
@@ -711,11 +711,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>elder_ray</t>
+          <t>mass_index</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>35.95</v>
+        <v>38.8</v>
       </c>
     </row>
     <row r="21">
@@ -726,11 +726,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>atr_breakout</t>
+          <t>ultimate_osc</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>35.15</v>
+        <v>37.49</v>
       </c>
     </row>
     <row r="22">
@@ -741,11 +741,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>tema</t>
+          <t>elder_ray</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>31.59</v>
+        <v>35.54</v>
       </c>
     </row>
     <row r="23">
@@ -756,11 +756,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>chandelier</t>
+          <t>williams_r</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>30.83</v>
+        <v>34.33</v>
       </c>
     </row>
     <row r="24">
@@ -771,11 +771,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>vwap</t>
+          <t>atr_breakout</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>30.01</v>
+        <v>32.87</v>
       </c>
     </row>
     <row r="25">
@@ -786,11 +786,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>klinger</t>
+          <t>chandelier</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>29.34</v>
+        <v>30.83</v>
       </c>
     </row>
     <row r="26">
@@ -801,11 +801,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>single_ma</t>
+          <t>mfi</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>29.24</v>
+        <v>29.78</v>
       </c>
     </row>
     <row r="27">
@@ -816,11 +816,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>dpo</t>
+          <t>tema</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>27.95</v>
+        <v>29.37</v>
       </c>
     </row>
     <row r="28">
@@ -831,11 +831,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>chaikin_vol</t>
+          <t>coppock</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>27.68</v>
+        <v>28.88</v>
       </c>
     </row>
     <row r="29">
@@ -846,11 +846,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>mass_index</t>
+          <t>dpo</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>27.33</v>
+        <v>27.95</v>
       </c>
     </row>
     <row r="30">
@@ -861,11 +861,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>vwma</t>
+          <t>vwap</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>26.78</v>
+        <v>27.81</v>
       </c>
     </row>
     <row r="31">
@@ -876,11 +876,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ultimate_osc</t>
+          <t>klinger</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>26.12</v>
+        <v>27.15</v>
       </c>
     </row>
     <row r="32">
@@ -891,11 +891,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>roc</t>
+          <t>single_ma</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25.95</v>
+        <v>26.68</v>
       </c>
     </row>
     <row r="33">
@@ -921,11 +921,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>vpt</t>
+          <t>roc</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>23.46</v>
+        <v>25.57</v>
       </c>
     </row>
     <row r="35">
@@ -936,11 +936,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ad_line</t>
+          <t>vwma</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>19.69</v>
+        <v>24.63</v>
       </c>
     </row>
     <row r="36">
@@ -951,11 +951,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>stochastic</t>
+          <t>rsi</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>19.63</v>
+        <v>24.28</v>
       </c>
     </row>
     <row r="37">
@@ -966,11 +966,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>mfi</t>
+          <t>vpt</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>19.05</v>
+        <v>21.37</v>
       </c>
     </row>
     <row r="38">
@@ -981,11 +981,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>coppock</t>
+          <t>ad_line</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>18.23</v>
+        <v>19.69</v>
       </c>
     </row>
     <row r="39">
@@ -996,11 +996,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>std_channel</t>
+          <t>pvi</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>18.16</v>
+        <v>19.23</v>
       </c>
     </row>
     <row r="40">
@@ -1011,11 +1011,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>cci</t>
+          <t>std_channel</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>15.12</v>
+        <v>18.16</v>
       </c>
     </row>
     <row r="41">
@@ -1026,11 +1026,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>rsi</t>
+          <t>stochastic</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>14</v>
+        <v>17.61</v>
       </c>
     </row>
     <row r="42">
@@ -1041,11 +1041,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>atr_channel</t>
+          <t>cci</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>11.58</v>
+        <v>15.12</v>
       </c>
     </row>
     <row r="43">
@@ -1056,11 +1056,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>schaff_trend</t>
+          <t>atr_channel</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>9.6</v>
+        <v>11.58</v>
       </c>
     </row>
     <row r="44">
@@ -1071,11 +1071,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>pvi</t>
+          <t>schaff_trend</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>9.380000000000001</v>
+        <v>7.75</v>
       </c>
     </row>
     <row r="45">
@@ -1116,11 +1116,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>momentum</t>
+          <t>rsi_divergence</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6.58</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="48">
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>6.42</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="49">
@@ -1146,11 +1146,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>stoch_rsi</t>
+          <t>bb_rsi</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2.01</v>
+        <v>5.27</v>
       </c>
     </row>
     <row r="50">
@@ -1161,11 +1161,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>hammer</t>
+          <t>momentum</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1.59</v>
+        <v>4.46</v>
       </c>
     </row>
     <row r="51">
@@ -1176,11 +1176,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>engulfing</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0.92</v>
+        <v>3.08</v>
       </c>
     </row>
     <row r="52">
@@ -1191,11 +1191,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>fractal_breakout</t>
+          <t>stoch_rsi</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.54</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="53">
@@ -1206,11 +1206,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>rsi_divergence</t>
+          <t>hammer</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>-2.39</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="54">
@@ -1221,11 +1221,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>three_ma</t>
+          <t>connors_rsi</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>-2.69</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="55">
@@ -1236,11 +1236,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>bb_rsi</t>
+          <t>engulfing</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>-3.43</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="56">
@@ -1251,11 +1251,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>cmf</t>
+          <t>squeeze</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>-3.68</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="57">
@@ -1266,11 +1266,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>awesome_oscillator</t>
+          <t>fractal_breakout</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>-3.88</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="58">
@@ -1281,11 +1281,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>zscore</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>-5.44</v>
+        <v>-0.44</v>
       </c>
     </row>
     <row r="59">
@@ -1296,11 +1296,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>connors_rsi</t>
+          <t>three_ma</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>-6.61</v>
+        <v>-2.69</v>
       </c>
     </row>
     <row r="60">
@@ -1311,11 +1311,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>two_ma</t>
+          <t>cmf</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>-7.11</v>
+        <v>-3.68</v>
       </c>
     </row>
     <row r="61">
@@ -1326,11 +1326,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>obv_ma</t>
+          <t>awesome_oscillator</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>-7.42</v>
+        <v>-3.88</v>
       </c>
     </row>
     <row r="62">
@@ -1341,11 +1341,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>squeeze</t>
+          <t>two_ma</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>-7.49</v>
+        <v>-7.11</v>
       </c>
     </row>
     <row r="63">
@@ -1356,11 +1356,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>adx</t>
+          <t>obv_ma</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>-9.220000000000001</v>
+        <v>-7.42</v>
       </c>
     </row>
     <row r="64">
@@ -1371,11 +1371,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>zscore</t>
+          <t>adx</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>-9.67</v>
+        <v>-9.220000000000001</v>
       </c>
     </row>
     <row r="65">
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>-18.91</v>
+        <v>-20.28</v>
       </c>
     </row>
     <row r="75">
@@ -1536,11 +1536,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>true_range_ema</t>
+          <t>trix</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>-22.28</v>
+        <v>-22.5</v>
       </c>
     </row>
     <row r="76">
@@ -1551,11 +1551,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>trix</t>
+          <t>hp_filter_ma</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>-22.5</v>
+        <v>-22.52</v>
       </c>
     </row>
     <row r="77">
@@ -1566,11 +1566,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>hp_filter_ma</t>
+          <t>true_range_ema</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>-22.52</v>
+        <v>-23.59</v>
       </c>
     </row>
     <row r="78">
@@ -1581,11 +1581,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>rvi</t>
+          <t>ichimoku</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>-23.5</v>
+        <v>-23.68</v>
       </c>
     </row>
     <row r="79">
@@ -1596,11 +1596,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ichimoku</t>
+          <t>wma</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>-23.68</v>
+        <v>-24.47</v>
       </c>
     </row>
     <row r="80">
@@ -1611,11 +1611,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>wma</t>
+          <t>bb_width</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>-24.47</v>
+        <v>-24.71</v>
       </c>
     </row>
     <row r="81">
@@ -1626,11 +1626,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>donchian</t>
+          <t>rvi</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>-25.36</v>
+        <v>-24.79</v>
       </c>
     </row>
     <row r="82">
@@ -1641,11 +1641,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>supertrend_rsi</t>
+          <t>donchian</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>-25.46</v>
+        <v>-25.36</v>
       </c>
     </row>
     <row r="83">
@@ -1656,11 +1656,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>inside_bar</t>
+          <t>supertrend_rsi</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>-29.01</v>
+        <v>-25.46</v>
       </c>
     </row>
     <row r="84">
@@ -1671,11 +1671,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>rsi_macd</t>
+          <t>vix_fix</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>-30.22</v>
+        <v>-26.55</v>
       </c>
     </row>
     <row r="85">
@@ -1686,11 +1686,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>bb_width</t>
+          <t>inside_bar</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>-30.93</v>
+        <v>-29.01</v>
       </c>
     </row>
     <row r="86">
@@ -1701,11 +1701,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>vix_fix</t>
+          <t>marubozu</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>-33.36</v>
+        <v>-29.05</v>
       </c>
     </row>
     <row r="87">
@@ -1716,11 +1716,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>marubozu</t>
+          <t>rsi_macd</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>-34.92</v>
+        <v>-30.22</v>
       </c>
     </row>
     <row r="88">
@@ -1780,7 +1780,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>-53.1</v>
+        <v>-48.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>